<commit_message>
Add 1h+ and 100K-views filter tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V9JS3ghqLfmLCFrdDWiZ2i
</commit_message>
<xml_diff>
--- a/faceless_horror_channels_ES_PT.xlsx
+++ b/faceless_horror_channels_ES_PT.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Qualified" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Maybe" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Excluded after checks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Method &amp; notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="1h+ &amp; 100K filter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Qualified" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Maybe" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Excluded after checks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Method &amp; notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -76,6 +77,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,226 +446,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Result: no channel meets BOTH 100K+ avg views AND mostly 1h+ videos while also being faceless, LatAm/Brazil, active ≤14 days and not on Spotify. Every ES/PT channel at that level is a podcast with hosts on camera, posts full movies, is English-language or is already on Spotify (checked ~3,300 channels incl. a new search of recent 1h+ videos sorted by views).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Channel name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Channel link</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Subscribers</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Average views (last 10 long videos)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Typical video length</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Last upload date</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Business email (from the About page, if listed)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>On Spotify? (Yes/No)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Language</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>EL IVANVILLA</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@elivanvilla</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>182K</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>162000</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>median 31 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Animated horror stories (1h+ compilations). Sister channel Elivanvilla2 is in Maybe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Mistere</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@Misterecore</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>97.8K</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>155900</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>median 38 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Dark mysteries / conspiracy (CIA experiments etc.). Faceless edits.</t>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Avg views (last 10 long)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Median length</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Videos ≥60 min (last 10)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Last upload</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>On Spotify?</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Ment3curiosa🧠</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@ment3curiosa-m2e</t>
+          <t>Closest to both</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Elivanvilla2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/@Elivanvilla98</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>Mexico</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>22.7K</t>
-        </is>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>150400</v>
+        <v>232700</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>median 49 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>50 min</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>5/10</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -670,52 +566,47 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Mystery icebergs (misterios de la humanidad, sociedades secretas).</t>
+          <t>Only miss: last upload 2026-09-06 (20 days). Animated horror, "1 HORA" compilations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Crimes Narrados</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@crimesnarrados02</t>
+          <t>1h+ videos (views 20–30K)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>HORROR SOBRENATURAL</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/@HorrorSobrenatural.Oficial</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>Brazil</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>12.9K</t>
-        </is>
-      </c>
       <c r="E5" s="4" t="n">
-        <v>135516</v>
+        <v>30200</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>median 43 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>82 min</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>10/10</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -725,52 +616,47 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>True crime narrated over photos; 12.9K subs but very high views.</t>
+          <t>All 10 recent videos ≥1h.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>O.Documentário</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@o.documentario</t>
+          <t>1h+ videos (views 20–30K)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>HISTORIAS DE HORROR Y FANTASÍA</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>https://www.youtube.com/@LADYHORRIDA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1.67K</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>51082</v>
+        <v>22400</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>median 52 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
+          <t>61 min</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>8/10</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -780,52 +666,47 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Dark Brazilian history: tragedies/disasters (Joelma fire, Bateau Mouche). 1.7K subs, recent videos breaking out.</t>
+          <t>8/10 ≥1h.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>El Laberinto del Misterio</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@ElLaberintodelMisterio-j8d</t>
+          <t>1h+ videos (views 20–30K)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Di Loreto Horror</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/@DiLoretoHorror</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>41.9K</t>
-        </is>
-      </c>
       <c r="E7" s="4" t="n">
-        <v>48450</v>
+        <v>23290</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>median 41 min · 9/10 ≥30 min · 2/10 ≥60 min</t>
+          <t>121 min</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>7/10</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -835,54 +716,49 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Unsolved mysteries / iceberg series ("Vol. 15").</t>
+          <t>7/10 ≥1h, median ~2h.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Historias Entre Paredes</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@Historias-entre-paredes</t>
+          <t>1h+ videos (views 20–30K)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Confesionario Oscuro</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>https://www.youtube.com/@ConfesionarioOscuro</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>7.87K</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>45685</v>
+        <v>25930</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>median 41 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>68 min</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>6/10</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>historiasentreparedes@gmail.com</t>
-        </is>
-      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -890,52 +766,47 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Dark-history / true-crime documentaries.</t>
+          <t>6/10 ≥1h.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cazador de Mentes</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@cazadordementes</t>
+          <t>100K+ views (videos 30–50 min)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EL IVANVILLA</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>https://www.youtube.com/@elivanvilla</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>38.6K</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>37900</v>
+        <v>162000</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>median 37 min · 8/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>31 min</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>0/10</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -945,52 +816,47 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Serial-killer true crime.</t>
+          <t>Animated horror.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>papupro777</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@sashslasher</t>
+          <t>100K+ views (videos 30–50 min)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Mistere</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>https://www.youtube.com/@Misterecore</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>4.91K</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>35310</v>
+        <v>155900</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>median 32 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>38 min</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>1/10</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1000,52 +866,47 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Creepypasta narrations; small channel (4.9K subs) with high views.</t>
+          <t>Dark mysteries.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Historias en la Oscuridad</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@Historias-enla-Oscuridad</t>
+          <t>100K+ views (videos 30–50 min)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Ment3curiosa🧠</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/@ment3curiosa-m2e</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>Mexico</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>6.66K</t>
-        </is>
-      </c>
       <c r="E11" s="4" t="n">
-        <v>33980</v>
+        <v>150400</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>median 43 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>49 min</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>0/10</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1055,52 +916,47 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Pueblo / immigrant horror relatos.</t>
+          <t>Mystery icebergs.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Alguien te observa en la oscuridad</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@teobserva</t>
+          <t>100K+ views (videos 30–50 min)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Crimes Narrados</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>https://www.youtube.com/@crimesnarrados02</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>277K</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>33300</v>
+        <v>135516</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>median 43 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>43 min</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>0/10</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>conejonegroteobserva@gmail.com</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1110,477 +966,46 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Rural horror relatos (3 relatos per video). Only a fan-made playlist exists on Spotify, no show.</t>
+          <t>True crime.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HORROR SOBRENATURAL</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@HorrorSobrenatural.Oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>13.2K</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>30200</v>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>median 82 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Relatos: night watchmen, police, military horror.</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Confesionario Oscuro</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@ConfesionarioOscuro</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>4.43K</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>25930</v>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>median 68 min · 10/10 ≥30 min · 6/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Possession / Ouija / "La Mano Peluda" cases; stylised AI imagery, no presenter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Historias Oscuras</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@HistoriasOscurass</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>22.9K</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>25430</v>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>median 59 min · 10/10 ≥30 min · 4/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Night-worker horror stories. Unrelated "Histórias Oscuras Podcast" (María Carapia) exists on Spotify — different creator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Seguidores de lo Extraño</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@SEGUIDORESDELOEXTRA%C3%91O</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>211K</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>24200</v>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>median 31 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Relatos de brujería (witchcraft stories). Thumbnails are suggestive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Di Loreto Horror</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@DiLoretoHorror</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>72.7K</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>23290</v>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>median 121 min · 9/10 ≥30 min · 7/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Creepypasta compilations, many 1h+.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Entre Misterios</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@EntreMisteriosYT</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>11K</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>22952</v>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>median 34 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Mystery listicles (10 misterios perturbadores...).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>HISTORIAS DE HORROR Y FANTASÍA</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@LADYHORRIDA</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>4.27K</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>22400</v>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>median 61 min · 10/10 ≥30 min · 8/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Nahual / trucker horror stories, mostly 1h+.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>ErickMa</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@erickmatruecrime</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>5.17K</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>22320</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>median 32 min · 5/10 ≥30 min · 4/10 ≥60 min</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Erickmanegocios@proton.me</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>True crime. Borderline on length: 5/10 last videos ≥30 min.</t>
-        </is>
-      </c>
+          <t>Would pass 1h+ but excluded:</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DESPACHO DEL CRIMEN (74K avg, 10/10 ≥1h) — last upload 2026-09-06; El último huésped (55K, 10/10 ≥1h) — on Spotify.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
-  </hyperlinks>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1660,19 +1085,19 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Why it is a Maybe</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Elivanvilla2</t>
+          <t>EL IVANVILLA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Elivanvilla98</t>
+          <t>https://www.youtube.com/@elivanvilla</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1682,20 +1107,20 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>95.3K</t>
+          <t>182K</t>
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>232700</v>
+        <v>162000</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>median 50 min · 6/10 ≥30 min · 5/10 ≥60 min</t>
+          <t>median 31 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1715,19 +1140,19 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Last long upload 2026-09-06 (20 days) — fails 14-day rule only. Sister channel of EL IVANVILLA.</t>
+          <t>Animated horror stories (1h+ compilations). Sister channel Elivanvilla2 is in Maybe.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Hora da Escuridão</t>
+          <t>Mistere</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@HoradaEscurid%C3%A3o</t>
+          <t>https://www.youtube.com/@Misterecore</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1737,20 +1162,20 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>62.7K</t>
+          <t>97.8K</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>90740</v>
+        <v>155900</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>median 42 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
+          <t>median 38 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1770,42 +1195,42 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Last upload 2026-09-07 (19 days) — fails 14-day rule only. Reddit horror stories.</t>
+          <t>Dark mysteries / conspiracy (CIA experiments etc.). Faceless edits.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DESPACHO DEL CRIMEN</t>
+          <t>Ment3curiosa🧠</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@DESPACHODELCRIMEN</t>
+          <t>https://www.youtube.com/@ment3curiosa-m2e</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>31K</t>
+          <t>22.7K</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>74200</v>
+        <v>150400</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>median 95 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
+          <t>median 49 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1825,42 +1250,42 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Last upload 2026-09-06 (20 days). Serial-killer marathons 1-2h, strong fit otherwise.</t>
+          <t>Mystery icebergs (misterios de la humanidad, sociedades secretas).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Acampamento Noturno</t>
+          <t>Crimes Narrados</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@AcampamentoNoturno</t>
+          <t>https://www.youtube.com/@crimesnarrados02</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3.13K</t>
+          <t>12.9K</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>25800</v>
+        <v>135516</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>median 77 min · 8/8 ≥30 min · 7/8 ≥60 min</t>
+          <t>median 43 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1880,42 +1305,42 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Last upload 2026-09-06 (20 days); country not listed. Campsite/forest horror relatos.</t>
+          <t>True crime narrated over photos; 12.9K subs but very high views.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Cruzada Hostil</t>
+          <t>O.Documentário</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@CruzadaHostil</t>
+          <t>https://www.youtube.com/@o.documentario</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>94.8K</t>
+          <t>1.67K</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>38200</v>
+        <v>51082</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>median 33 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>median 52 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1930,52 +1355,52 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Last upload 2026-09-11 (15 days, one day over). Mafia documentaries using archival footage.</t>
+          <t>Dark Brazilian history: tragedies/disasters (Joelma fire, Bateau Mouche). 1.7K subs, recent videos breaking out.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bruno Villas</t>
+          <t>El Laberinto del Misterio</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@BrunoVillas</t>
+          <t>https://www.youtube.com/@ElLaberintodelMisterio-j8d</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>362K</t>
+          <t>41.9K</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>151600</v>
+        <v>48450</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>median 38 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 41 min · 9/10 ≥30 min · 2/10 ≥60 min</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>contato@brunovillas.com</t>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1985,52 +1410,52 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Last upload 2026-09-11 (15 days). True crime; thumbnails show no host but channel is named after a person — confirm he is not on camera.</t>
+          <t>Unsolved mysteries / iceberg series ("Vol. 15").</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tess Historias</t>
+          <t>Historias Entre Paredes</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@tesshistorias</t>
+          <t>https://www.youtube.com/@Historias-entre-paredes</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>18.4K</t>
+          <t>7.87K</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>93800</v>
+        <v>45685</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>median 49 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 41 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>historiasentreparedes@gmail.com</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -2045,42 +1470,42 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Passes numbers. Sister of "Tess Investiga" (host on camera); this channel's thumbnails show no host, but could not confirm she stays off camera.</t>
+          <t>Dark-history / true-crime documentaries.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Etheria Paranormal</t>
+          <t>Cazador de Mentes</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@EtheriaParanormal</t>
+          <t>https://www.youtube.com/@cazadordementes</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>112K</t>
+          <t>38.6K</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>130900</v>
+        <v>37900</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>median 45 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>median 37 min · 8/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -2100,47 +1525,47 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>"Historias paranormales contadas por sus protagonistas" — no presenter, but interviewees appear on camera. Last upload 2026-09-10 (16 days).</t>
+          <t>Serial-killer true crime.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FFF Escena Del Crimen | Pelis y Series Policíacas</t>
+          <t>papupro777</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@FFFEscenaDelCrimen</t>
+          <t>https://www.youtube.com/@sashslasher</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>48.3K</t>
+          <t>4.91K</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>59780</v>
+        <v>35310</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>median 47 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 32 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>info@greaterfool.tv</t>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -2155,47 +1580,47 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Full episodes of licensed/dubbed TV crime series (Los Fiscales, Los Nuevos Detectives); network channel (greaterfool.tv). Likely fails the reupload/TV rule.</t>
+          <t>Creepypasta narrations; small channel (4.9K subs) with high views.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>FFF Escena Del Misterio | Investigación Paranormal</t>
+          <t>Historias en la Oscuridad</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@FFFEscenaDelMisterio</t>
+          <t>https://www.youtube.com/@Historias-enla-Oscuridad</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>24.7K</t>
+          <t>6.66K</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>61930</v>
+        <v>33980</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>median 42 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 43 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>info@greaterfool.tv</t>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -2210,47 +1635,47 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Same network as above; licensed paranormal TV series. Likely fails the reupload/TV rule.</t>
+          <t>Pueblo / immigrant horror relatos.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Penguinator</t>
+          <t>Alguien te observa en la oscuridad</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Penguinatory</t>
+          <t>https://www.youtube.com/@teobserva</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>203K</t>
+          <t>277K</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>171100</v>
+        <v>33300</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>median 39 min · 10/10 ≥30 min · 3/10 ≥60 min</t>
+          <t>median 43 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>conejonegroteobserva@gmail.com</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2265,19 +1690,19 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Faceless, but "caught on camera" compilations of other people's footage.</t>
+          <t>Rural horror relatos (3 relatos per video). Only a fan-made playlist exists on Spotify, no show.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Mr. Haunted</t>
+          <t>HORROR SOBRENATURAL</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Mr.Assombrado</t>
+          <t>https://www.youtube.com/@HorrorSobrenatural.Oficial</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2287,25 +1712,25 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>237K</t>
+          <t>13.2K</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>72700</v>
+        <v>30200</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>median 32 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 82 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>mrhauntedvideos@gmail.com</t>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -2320,37 +1745,37 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Faceless found-footage compilations (others' clips).</t>
+          <t>Relatos: night watchmen, police, military horror.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Zona Do MEDO</t>
+          <t>Confesionario Oscuro</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@ZonaDoMEDO_Br</t>
+          <t>https://www.youtube.com/@ConfesionarioOscuro</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>63.1K</t>
+          <t>4.43K</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>53000</v>
+        <v>25930</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>median 34 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 68 min · 10/10 ≥30 min · 6/10 ≥60 min</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2370,42 +1795,42 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Faceless found-footage compilations (others' clips).</t>
+          <t>Possession / Ouija / "La Mano Peluda" cases; stylised AI imagery, no presenter.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Relato Mafioso</t>
+          <t>Historias Oscuras</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@RelatoMafioso</t>
+          <t>https://www.youtube.com/@HistoriasOscurass</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>73.8K</t>
+          <t>22.9K</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>19460</v>
+        <v>25430</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>median 47 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>median 59 min · 10/10 ≥30 min · 4/10 ≥60 min</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2430,42 +1855,42 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Avg 19,460 — just under 20K. Mafia/cartel true crime.</t>
+          <t>Night-worker horror stories. Unrelated "Histórias Oscuras Podcast" (María Carapia) exists on Spotify — different creator.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Relato de Casos Criminais</t>
+          <t>Seguidores de lo Extraño</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@relatodecasoscriminais</t>
+          <t>https://www.youtube.com/@SEGUIDORESDELOEXTRA%C3%91O</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>110K</t>
+          <t>211K</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>17580</v>
+        <v>24200</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>median 34 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
+          <t>median 31 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2480,47 +1905,47 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Avg 17,580 — under 20K; some thumbnails may show a presenter.</t>
+          <t>Relatos de brujería (witchcraft stories). Thumbnails are suggestive.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Rádio Noturno</t>
+          <t>Di Loreto Horror</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@radio.noturno</t>
+          <t>https://www.youtube.com/@DiLoretoHorror</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>6.7K</t>
+          <t>72.7K</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>16420</v>
+        <v>23290</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>median 53 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
+          <t>median 121 min · 9/10 ≥30 min · 7/10 ≥60 min</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2535,47 +1960,47 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Avg 16,420 and last upload 2026-09-06. Urban legends / 3-hour compilations.</t>
+          <t>Creepypasta compilations, many 1h+.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Terror Macabro</t>
+          <t>Entre Misterios</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@terrormacabro_</t>
+          <t>https://www.youtube.com/@EntreMisteriosYT</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>34.5K</t>
+          <t>11K</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>13810</v>
+        <v>22952</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>median 34 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 34 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2590,47 +2015,47 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Avg 13,810 — under 20K. Relatos de terror, 1h format.</t>
+          <t>Mystery listicles (10 misterios perturbadores...).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Expediente Oscuro</t>
+          <t>HISTORIAS DE HORROR Y FANTASÍA</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@ExpedienteOscuroDoc</t>
+          <t>https://www.youtube.com/@LADYHORRIDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>6.43K</t>
+          <t>4.27K</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>13610</v>
+        <v>22400</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>median 70 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
+          <t>median 61 min · 10/10 ≥30 min · 8/10 ≥60 min</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2650,47 +2075,47 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Avg 13,610 — under 20K. True crime compilations.</t>
+          <t>Nahual / trucker horror stories, mostly 1h+.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Ecos de lo Macabro</t>
+          <t>ErickMa</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@EcosdeloMacabro</t>
+          <t>https://www.youtube.com/@erickmatruecrime</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>33K</t>
+          <t>5.17K</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>11860</v>
+        <v>22320</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>median 35 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+          <t>median 32 min · 5/10 ≥30 min · 4/10 ≥60 min</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+          <t>Erickmanegocios@proton.me</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2705,7 +2130,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Avg 11,860 — under 20K. Rancho/hospital horror.</t>
+          <t>True crime. Borderline on length: 5/10 last videos ≥30 min.</t>
         </is>
       </c>
     </row>
@@ -2736,6 +2161,1156 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Channel name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Channel link</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Subscribers</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Average views (last 10 long videos)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Typical video length</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Last upload date</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Business email (from the About page, if listed)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>On Spotify? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Why it is a Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Elivanvilla2</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@Elivanvilla98</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>95.3K</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>232700</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>median 50 min · 6/10 ≥30 min · 5/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Last long upload 2026-09-06 (20 days) — fails 14-day rule only. Sister channel of EL IVANVILLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Hora da Escuridão</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@HoradaEscurid%C3%A3o</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>62.7K</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>90740</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>median 42 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Last upload 2026-09-07 (19 days) — fails 14-day rule only. Reddit horror stories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DESPACHO DEL CRIMEN</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@DESPACHODELCRIMEN</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>31K</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>74200</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>median 95 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Last upload 2026-09-06 (20 days). Serial-killer marathons 1-2h, strong fit otherwise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Acampamento Noturno</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@AcampamentoNoturno</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>3.13K</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>25800</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>median 77 min · 8/8 ≥30 min · 7/8 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Last upload 2026-09-06 (20 days); country not listed. Campsite/forest horror relatos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Cruzada Hostil</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@CruzadaHostil</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>94.8K</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>38200</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>median 33 min · 8/10 ≥30 min · 1/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Last upload 2026-09-11 (15 days, one day over). Mafia documentaries using archival footage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Bruno Villas</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@BrunoVillas</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>362K</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>151600</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>median 38 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>contato@brunovillas.com</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Last upload 2026-09-11 (15 days). True crime; thumbnails show no host but channel is named after a person — confirm he is not on camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Tess Historias</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@tesshistorias</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>18.4K</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>93800</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>median 49 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Passes numbers. Sister of "Tess Investiga" (host on camera); this channel's thumbnails show no host, but could not confirm she stays off camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Etheria Paranormal</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@EtheriaParanormal</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>112K</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>130900</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>median 45 min · 9/10 ≥30 min · 1/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>"Historias paranormales contadas por sus protagonistas" — no presenter, but interviewees appear on camera. Last upload 2026-09-10 (16 days).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>FFF Escena Del Crimen | Pelis y Series Policíacas</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@FFFEscenaDelCrimen</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>48.3K</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>59780</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>median 47 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>info@greaterfool.tv</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Full episodes of licensed/dubbed TV crime series (Los Fiscales, Los Nuevos Detectives); network channel (greaterfool.tv). Likely fails the reupload/TV rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>FFF Escena Del Misterio | Investigación Paranormal</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@FFFEscenaDelMisterio</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>24.7K</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>61930</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>median 42 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>info@greaterfool.tv</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Same network as above; licensed paranormal TV series. Likely fails the reupload/TV rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Penguinator</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@Penguinatory</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>203K</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>171100</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>median 39 min · 10/10 ≥30 min · 3/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Faceless, but "caught on camera" compilations of other people's footage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Haunted</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@Mr.Assombrado</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>237K</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>72700</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>median 32 min · 6/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>mrhauntedvideos@gmail.com</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Faceless found-footage compilations (others' clips).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Zona Do MEDO</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@ZonaDoMEDO_Br</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>63.1K</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>53000</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>median 34 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Faceless found-footage compilations (others' clips).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Relato Mafioso</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@RelatoMafioso</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>73.8K</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>19460</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>median 47 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Avg 19,460 — just under 20K. Mafia/cartel true crime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Relato de Casos Criminais</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@relatodecasoscriminais</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>110K</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>17580</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>median 34 min · 8/10 ≥30 min · 2/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Avg 17,580 — under 20K; some thumbnails may show a presenter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Rádio Noturno</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@radio.noturno</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>6.7K</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>16420</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>median 53 min · 10/10 ≥30 min · 1/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Avg 16,420 and last upload 2026-09-06. Urban legends / 3-hour compilations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Terror Macabro</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@terrormacabro_</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>34.5K</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>13810</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>median 34 min · 10/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Avg 13,810 — under 20K. Relatos de terror, 1h format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Expediente Oscuro</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@ExpedienteOscuroDoc</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>6.43K</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>13610</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>median 70 min · 10/10 ≥30 min · 10/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Avg 13,610 — under 20K. True crime compilations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Ecos de lo Macabro</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@EcosdeloMacabro</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>33K</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>11860</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>median 35 min · 9/10 ≥30 min · 0/10 ≥60 min</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Not listed publicly (About-page email button needs sign-in; check manually)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Avg 11,860 — under 20K. Rancho/hospital horror.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3690,7 +4265,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>